<commit_message>
Add charts, LULU memo, Streamlit app, and README results section
- dcf/charts.py: margin, tornado and scenario charts, written by the CLI
- docs/LULU_memo.md and PDF, built with scripts/build_memo.py
- app.py: Streamlit front end with assumption sliders and workbook download
- README leads with the LULU result and links to the memo and model
- Clear errors when the SEC rejects the User-Agent or core 10-K figures are missing
</commit_message>
<xml_diff>
--- a/output/LULU_dcf.xlsx
+++ b/output/LULU_dcf.xlsx
@@ -570,7 +570,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Base period TTM Aug-26 (ended 02 Aug 2026). Market data as of 2026-10-20. Blue = input (edit freely); black = formula.</t>
+          <t>Base period TTM Aug-26 (ended 02 Aug 2026). Market data as of 2026-10-23. Blue = input (edit freely); black = formula.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>99.94000244140625</v>
+        <v>99.01000213623047</v>
       </c>
     </row>
     <row r="6">
@@ -2046,10 +2046,10 @@
         <v>0.03</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>-0.1265361560942988</v>
+        <v>-0.1301220543509444</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>-0.04603776902853529</v>
+        <v>-0.04751228246399886</v>
       </c>
     </row>
     <row r="6">
@@ -2062,7 +2062,7 @@
         <v>0.17</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.1053995961913747</v>
+        <v>0.1042572125430389</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>0.01705837228896923</v>
@@ -2076,7 +2076,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Price used: $99.94 as of 2026-10-20</t>
+          <t>Price used: $99.01 as of 2026-10-23</t>
         </is>
       </c>
       <c r="B8" s="2" t="n"/>
@@ -2532,7 +2532,7 @@
         <v>115.3624524547555</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>0.1543170866179562</v>
+        <v>0.1651595794940521</v>
       </c>
       <c r="F24" s="10" t="n">
         <v>0.25</v>
@@ -2554,7 +2554,7 @@
         <v>152.5303868923924</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>0.5262195634007447</v>
+        <v>0.5405553338189191</v>
       </c>
       <c r="F25" s="10" t="n">
         <v>0.5</v>
@@ -2576,7 +2576,7 @@
         <v>198.4516557628887</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>0.9857079339100359</v>
+        <v>1.004359675599581</v>
       </c>
       <c r="F26" s="10" t="n">
         <v>0.25</v>

</xml_diff>